<commit_message>
updated admin panel and optimized code
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -424,10 +424,10 @@
         <v>Nordic Chair</v>
       </c>
       <c r="C2" t="str">
-        <v>A sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chairA sleek nordic style chair</v>
+        <v>hdjahdbasjdsh</v>
       </c>
       <c r="D2" t="str">
-        <v>blockfixo</v>
+        <v>Tile Spacer</v>
       </c>
       <c r="E2" t="str">
         <v>images\person_1.jpg</v>

</xml_diff>